<commit_message>
Actualizacion de la vision de cobertura de alimentos en crosswalk_variedad_INCAP.xlsx  3 pm 24/08/2016.md
</commit_message>
<xml_diff>
--- a/data/raw/crosswalk_variedad_INCAP.xlsx
+++ b/data/raw/crosswalk_variedad_INCAP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wfp-my.sharepoint.com/personal/maicel_monzon_wfp_org/Documents/Documents/Fases_Consultoria/01_analisis_ENGIH2018/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="368" documentId="14_{F8BE0E5F-76BA-446B-8942-BC5680A971A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA8EAFD1-C70C-4AC1-B63F-C5D263252057}"/>
+  <xr:revisionPtr revIDLastSave="454" documentId="14_{F8BE0E5F-76BA-446B-8942-BC5680A971A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF0E0AF7-0E0D-4AC1-AD13-F9A3A744D940}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Datos" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Datos!$A$1:$S$773</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Datos!$A$1:$R$773</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5006" uniqueCount="2232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5019" uniqueCount="2232">
   <si>
     <t>Cómo usar este archivo</t>
   </si>
@@ -6892,7 +6892,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6944,6 +6944,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7617,9 +7620,9 @@
   <dimension ref="A1:R773"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.1796875" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="32.54296875" customWidth="1"/>
-    <col min="3" max="3" width="14.08984375" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="14.08984375" customWidth="1"/>
     <col min="4" max="4" width="21.81640625" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="14.6328125" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="24.54296875" hidden="1" customWidth="1"/>
@@ -7627,7 +7630,7 @@
     <col min="8" max="8" width="18" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="9.453125" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="17.81640625" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.7265625" customWidth="1"/>
     <col min="12" max="12" width="20.36328125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20" customWidth="1"/>
@@ -7644,7 +7647,7 @@
       <c r="B1" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="26" t="s">
         <v>28</v>
       </c>
       <c r="D1" s="11" t="s">
@@ -12548,10 +12551,14 @@
       <c r="H96" s="14"/>
       <c r="I96" s="14"/>
       <c r="J96" s="14"/>
-      <c r="K96" s="15"/>
-      <c r="L96" s="15"/>
+      <c r="K96" s="15">
+        <v>70201032</v>
+      </c>
+      <c r="L96" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M96" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N96" s="15"/>
       <c r="O96" s="16" t="s">
@@ -15350,10 +15357,14 @@
       <c r="H159" s="14"/>
       <c r="I159" s="14"/>
       <c r="J159" s="14"/>
-      <c r="K159" s="15"/>
-      <c r="L159" s="15"/>
+      <c r="K159" s="15">
+        <v>70201103</v>
+      </c>
+      <c r="L159" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M159" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N159" s="15"/>
       <c r="O159" s="16" t="s">
@@ -15840,10 +15851,14 @@
       <c r="H170" s="14"/>
       <c r="I170" s="14"/>
       <c r="J170" s="14"/>
-      <c r="K170" s="15"/>
-      <c r="L170" s="15"/>
+      <c r="K170" s="15">
+        <v>70201083</v>
+      </c>
+      <c r="L170" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M170" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N170" s="15"/>
       <c r="O170" s="16" t="s">
@@ -16724,10 +16739,14 @@
       <c r="H190" s="14"/>
       <c r="I190" s="14"/>
       <c r="J190" s="14"/>
-      <c r="K190" s="15"/>
-      <c r="L190" s="15"/>
+      <c r="K190" s="15">
+        <v>70201009</v>
+      </c>
+      <c r="L190" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M190" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N190" s="15"/>
       <c r="O190" s="16" t="s">
@@ -18408,10 +18427,14 @@
       <c r="H228" s="14"/>
       <c r="I228" s="14"/>
       <c r="J228" s="14"/>
-      <c r="K228" s="15"/>
-      <c r="L228" s="15"/>
+      <c r="K228" s="15">
+        <v>70201008</v>
+      </c>
+      <c r="L228" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M228" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N228" s="15"/>
       <c r="O228" s="16" t="s">
@@ -20840,10 +20863,14 @@
       <c r="H283" s="14"/>
       <c r="I283" s="14"/>
       <c r="J283" s="14"/>
-      <c r="K283" s="15"/>
-      <c r="L283" s="15"/>
+      <c r="K283" s="15">
+        <v>70201086</v>
+      </c>
+      <c r="L283" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M283" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N283" s="15"/>
       <c r="O283" s="16" t="s">
@@ -21192,10 +21219,14 @@
       <c r="H291" s="14"/>
       <c r="I291" s="14"/>
       <c r="J291" s="14"/>
-      <c r="K291" s="15"/>
-      <c r="L291" s="15"/>
+      <c r="K291" s="15">
+        <v>70201026</v>
+      </c>
+      <c r="L291" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M291" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N291" s="15"/>
       <c r="O291" s="16" t="s">
@@ -27140,10 +27171,14 @@
       <c r="H425" s="14"/>
       <c r="I425" s="14"/>
       <c r="J425" s="14"/>
-      <c r="K425" s="15"/>
-      <c r="L425" s="15"/>
+      <c r="K425" s="15">
+        <v>70201105</v>
+      </c>
+      <c r="L425" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M425" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N425" s="15"/>
       <c r="O425" s="16" t="s">
@@ -30866,10 +30901,14 @@
       <c r="H509" s="14"/>
       <c r="I509" s="14"/>
       <c r="J509" s="14"/>
-      <c r="K509" s="15"/>
-      <c r="L509" s="15"/>
+      <c r="K509" s="15">
+        <v>70201052</v>
+      </c>
+      <c r="L509" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M509" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N509" s="15"/>
       <c r="O509" s="16" t="s">
@@ -31310,10 +31349,14 @@
       <c r="H519" s="14"/>
       <c r="I519" s="14"/>
       <c r="J519" s="14"/>
-      <c r="K519" s="15"/>
-      <c r="L519" s="15"/>
+      <c r="K519" s="15">
+        <v>70201119</v>
+      </c>
+      <c r="L519" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M519" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N519" s="15"/>
       <c r="O519" s="16" t="s">
@@ -33706,10 +33749,14 @@
       <c r="H573" s="14"/>
       <c r="I573" s="14"/>
       <c r="J573" s="14"/>
-      <c r="K573" s="15"/>
-      <c r="L573" s="15"/>
+      <c r="K573" s="15">
+        <v>70201010</v>
+      </c>
+      <c r="L573" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M573" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N573" s="15"/>
       <c r="O573" s="16" t="s">
@@ -37230,10 +37277,14 @@
       <c r="H653" s="14"/>
       <c r="I653" s="14"/>
       <c r="J653" s="14"/>
-      <c r="K653" s="15"/>
-      <c r="L653" s="15"/>
+      <c r="K653" s="15">
+        <v>70201015</v>
+      </c>
+      <c r="L653" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M653" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N653" s="15"/>
       <c r="O653" s="16" t="s">
@@ -42100,10 +42151,14 @@
       <c r="H763" s="14"/>
       <c r="I763" s="14"/>
       <c r="J763" s="14"/>
-      <c r="K763" s="15"/>
-      <c r="L763" s="15"/>
+      <c r="K763" s="15">
+        <v>70201103</v>
+      </c>
+      <c r="L763" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M763" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N763" s="15"/>
       <c r="O763" s="16" t="s">
@@ -42560,7 +42615,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S773" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:R773" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <conditionalFormatting sqref="B2:B773">
     <cfRule type="expression" dxfId="4" priority="5">
       <formula>$H2&lt;&gt;""</formula>

</xml_diff>

<commit_message>
Actualizacion de la vision de cobertura de alimentos en crosswalk_variedad_INCAP.xlsx  4 pm 24/08/2016.md
</commit_message>
<xml_diff>
--- a/data/raw/crosswalk_variedad_INCAP.xlsx
+++ b/data/raw/crosswalk_variedad_INCAP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wfp-my.sharepoint.com/personal/maicel_monzon_wfp_org/Documents/Documents/Fases_Consultoria/01_analisis_ENGIH2018/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="454" documentId="14_{F8BE0E5F-76BA-446B-8942-BC5680A971A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF0E0AF7-0E0D-4AC1-AD13-F9A3A744D940}"/>
+  <xr:revisionPtr revIDLastSave="516" documentId="14_{F8BE0E5F-76BA-446B-8942-BC5680A971A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B86A18F-06E1-4855-8336-057BAE4CE478}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5019" uniqueCount="2232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5031" uniqueCount="2232">
   <si>
     <t>Cómo usar este archivo</t>
   </si>
@@ -7623,12 +7623,12 @@
     <col min="1" max="1" width="14.1796875" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="32.54296875" customWidth="1"/>
     <col min="3" max="3" width="14.08984375" customWidth="1"/>
-    <col min="4" max="4" width="21.81640625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="21.81640625" customWidth="1"/>
     <col min="5" max="5" width="14.6328125" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="24.54296875" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="23.453125" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="18" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="9.453125" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="9.453125" customWidth="1"/>
     <col min="10" max="10" width="17.81640625" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="16.7265625" customWidth="1"/>
     <col min="12" max="12" width="20.36328125" bestFit="1" customWidth="1"/>
@@ -7650,7 +7650,7 @@
       <c r="C1" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="26" t="s">
         <v>30</v>
       </c>
       <c r="E1" s="11" t="s">
@@ -7833,10 +7833,14 @@
       <c r="J4" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
+      <c r="K4" s="14">
+        <v>70203019</v>
+      </c>
+      <c r="L4" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M4" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" s="15"/>
       <c r="O4" s="16" t="s">
@@ -7939,7 +7943,7 @@
         <v>94</v>
       </c>
       <c r="K6" s="15">
-        <f t="shared" ref="K6:K8" si="0">I6</f>
+        <f>I6</f>
         <v>70202002</v>
       </c>
       <c r="L6" s="15" t="s">
@@ -7994,7 +7998,7 @@
         <v>99</v>
       </c>
       <c r="K7" s="15">
-        <f t="shared" si="0"/>
+        <f>I7</f>
         <v>70211006</v>
       </c>
       <c r="L7" s="15" t="s">
@@ -8051,7 +8055,7 @@
         <v>99</v>
       </c>
       <c r="K8" s="15">
-        <f t="shared" si="0"/>
+        <f>I8</f>
         <v>70216009</v>
       </c>
       <c r="L8" s="15" t="s">
@@ -8105,10 +8109,14 @@
       <c r="J9" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
+      <c r="K9" s="14">
+        <v>70214021</v>
+      </c>
+      <c r="L9" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M9" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N9" s="15"/>
       <c r="O9" s="16" t="s">
@@ -8155,10 +8163,14 @@
       <c r="J10" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="K10" s="15"/>
-      <c r="L10" s="15"/>
+      <c r="K10" s="15">
+        <v>70217063</v>
+      </c>
+      <c r="L10" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M10" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N10" s="15"/>
       <c r="O10" s="16" t="s">
@@ -8259,10 +8271,14 @@
       <c r="J12" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="K12" s="15"/>
-      <c r="L12" s="15"/>
+      <c r="K12" s="14">
+        <v>70222047</v>
+      </c>
+      <c r="L12" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M12" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N12" s="15"/>
       <c r="O12" s="16" t="s">
@@ -8364,7 +8380,7 @@
         <v>137</v>
       </c>
       <c r="K14" s="15">
-        <f t="shared" ref="K14:K15" si="1">I14</f>
+        <f>I14</f>
         <v>70217039</v>
       </c>
       <c r="L14" s="15" t="s">
@@ -8421,7 +8437,7 @@
         <v>143</v>
       </c>
       <c r="K15" s="15">
-        <f t="shared" si="1"/>
+        <f>I15</f>
         <v>70215003</v>
       </c>
       <c r="L15" s="15" t="s">
@@ -8526,7 +8542,7 @@
         <v>153</v>
       </c>
       <c r="K17" s="15">
-        <f t="shared" ref="K17:K18" si="2">I17</f>
+        <f>I17</f>
         <v>70213004</v>
       </c>
       <c r="L17" s="15" t="s">
@@ -8581,7 +8597,7 @@
         <v>99</v>
       </c>
       <c r="K18" s="15">
-        <f t="shared" si="2"/>
+        <f>I18</f>
         <v>70212131</v>
       </c>
       <c r="L18" s="15" t="s">
@@ -8635,10 +8651,14 @@
       <c r="J19" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="K19" s="15"/>
-      <c r="L19" s="15"/>
+      <c r="K19" s="14">
+        <v>70214112</v>
+      </c>
+      <c r="L19" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M19" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19" s="15"/>
       <c r="O19" s="16" t="s">
@@ -8686,7 +8706,7 @@
         <v>99</v>
       </c>
       <c r="K20" s="15">
-        <f t="shared" ref="K20" si="3">I20</f>
+        <f>I20</f>
         <v>70212011</v>
       </c>
       <c r="L20" s="15" t="s">
@@ -8740,10 +8760,14 @@
       <c r="J21" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="K21" s="15"/>
-      <c r="L21" s="15"/>
+      <c r="K21" s="14">
+        <v>70222022</v>
+      </c>
+      <c r="L21" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M21" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N21" s="15"/>
       <c r="O21" s="16" t="s">
@@ -8790,10 +8814,14 @@
       <c r="J22" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
+      <c r="K22" s="15">
+        <v>70207037</v>
+      </c>
+      <c r="L22" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M22" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="15"/>
       <c r="O22" s="16" t="s">
@@ -8841,7 +8869,7 @@
         <v>99</v>
       </c>
       <c r="K23" s="15">
-        <f t="shared" ref="K23:K24" si="4">I23</f>
+        <f>I23</f>
         <v>70211167</v>
       </c>
       <c r="L23" s="15" t="s">
@@ -8896,7 +8924,7 @@
         <v>186</v>
       </c>
       <c r="K24" s="15">
-        <f t="shared" si="4"/>
+        <f>I24</f>
         <v>70201015</v>
       </c>
       <c r="L24" s="15" t="s">
@@ -8950,10 +8978,14 @@
       <c r="J25" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15"/>
+      <c r="K25" s="15">
+        <v>70214009</v>
+      </c>
+      <c r="L25" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M25" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N25" s="15"/>
       <c r="O25" s="16" t="s">
@@ -9000,10 +9032,14 @@
       <c r="J26" s="14" t="s">
         <v>197</v>
       </c>
-      <c r="K26" s="15"/>
-      <c r="L26" s="15"/>
+      <c r="K26" s="24">
+        <v>70211127</v>
+      </c>
+      <c r="L26" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M26" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N26" s="15"/>
       <c r="O26" s="16" t="s">
@@ -9051,7 +9087,7 @@
         <v>202</v>
       </c>
       <c r="K27" s="15">
-        <f t="shared" ref="K27:K28" si="5">I27</f>
+        <f>I27</f>
         <v>70209006</v>
       </c>
       <c r="L27" s="15" t="s">
@@ -9106,7 +9142,7 @@
         <v>207</v>
       </c>
       <c r="K28" s="15">
-        <f t="shared" si="5"/>
+        <f>I28</f>
         <v>70201014</v>
       </c>
       <c r="L28" s="15" t="s">
@@ -9215,7 +9251,7 @@
         <v>216</v>
       </c>
       <c r="K30" s="15">
-        <f t="shared" ref="K30:K32" si="6">I30</f>
+        <f>I30</f>
         <v>70212107</v>
       </c>
       <c r="L30" s="15" t="s">
@@ -9270,7 +9306,7 @@
         <v>221</v>
       </c>
       <c r="K31" s="15">
-        <f t="shared" si="6"/>
+        <f>I31</f>
         <v>70211005</v>
       </c>
       <c r="L31" s="15" t="s">
@@ -9325,7 +9361,7 @@
         <v>226</v>
       </c>
       <c r="K32" s="15">
-        <f t="shared" si="6"/>
+        <f>I32</f>
         <v>70211157</v>
       </c>
       <c r="L32" s="15" t="s">
@@ -9485,10 +9521,14 @@
       <c r="J35" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="K35" s="15"/>
-      <c r="L35" s="15"/>
+      <c r="K35" s="24">
+        <v>70214004</v>
+      </c>
+      <c r="L35" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="M35" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N35" s="15"/>
       <c r="O35" s="16" t="s">
@@ -9592,7 +9632,7 @@
         <v>250</v>
       </c>
       <c r="K37" s="15">
-        <f t="shared" ref="K37" si="7">I37</f>
+        <f>I37</f>
         <v>70201052</v>
       </c>
       <c r="L37" s="15" t="s">
@@ -9758,7 +9798,7 @@
         <v>70217063</v>
       </c>
       <c r="L40" s="15" t="s">
-        <v>211</v>
+        <v>80</v>
       </c>
       <c r="M40" s="15" t="b">
         <v>1</v>
@@ -9827,17 +9867,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:18" s="21" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="14">
         <v>262</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B42" s="20" t="s">
         <v>270</v>
       </c>
-      <c r="C42" s="14">
+      <c r="C42" s="20">
         <v>1770</v>
       </c>
-      <c r="D42" s="14" t="s">
+      <c r="D42" s="20" t="s">
         <v>63</v>
       </c>
       <c r="E42" s="14">
@@ -9850,24 +9890,28 @@
         <v>185</v>
       </c>
       <c r="H42" s="14"/>
-      <c r="I42" s="14"/>
+      <c r="I42" s="20"/>
       <c r="J42" s="14"/>
-      <c r="K42" s="15"/>
-      <c r="L42" s="15"/>
-      <c r="M42" s="15" t="b">
-        <v>0</v>
-      </c>
-      <c r="N42" s="15"/>
-      <c r="O42" s="16" t="s">
+      <c r="K42" s="20">
+        <v>70201029</v>
+      </c>
+      <c r="L42" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="M42" s="20" t="b">
+        <v>1</v>
+      </c>
+      <c r="N42" s="20"/>
+      <c r="O42" s="20" t="s">
         <v>251</v>
       </c>
-      <c r="P42" s="16" t="s">
+      <c r="P42" s="20" t="s">
         <v>272</v>
       </c>
-      <c r="Q42" s="16">
+      <c r="Q42" s="20">
         <v>70.599999999999994</v>
       </c>
-      <c r="R42" s="16" t="b">
+      <c r="R42" s="20" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10193,7 +10237,7 @@
         <v>299</v>
       </c>
       <c r="K49" s="15">
-        <f t="shared" ref="K49" si="8">I49</f>
+        <f>I49</f>
         <v>70222005</v>
       </c>
       <c r="L49" s="15" t="s">
@@ -10406,7 +10450,7 @@
         <v>318</v>
       </c>
       <c r="K53" s="15">
-        <f t="shared" ref="K53:K56" si="9">I53</f>
+        <f>I53</f>
         <v>70211023</v>
       </c>
       <c r="L53" s="15" t="s">
@@ -10461,7 +10505,7 @@
         <v>323</v>
       </c>
       <c r="K54" s="15">
-        <f t="shared" si="9"/>
+        <f>I54</f>
         <v>70212103</v>
       </c>
       <c r="L54" s="15" t="s">
@@ -10516,7 +10560,7 @@
         <v>327</v>
       </c>
       <c r="K55" s="15">
-        <f t="shared" si="9"/>
+        <f>I55</f>
         <v>70209050</v>
       </c>
       <c r="L55" s="15" t="s">
@@ -10571,7 +10615,7 @@
         <v>330</v>
       </c>
       <c r="K56" s="15">
-        <f t="shared" si="9"/>
+        <f>I56</f>
         <v>70212010</v>
       </c>
       <c r="L56" s="15" t="s">
@@ -10680,7 +10724,7 @@
         <v>339</v>
       </c>
       <c r="K58" s="15">
-        <f t="shared" ref="K58" si="10">I58</f>
+        <f>I58</f>
         <v>70211169</v>
       </c>
       <c r="L58" s="15" t="s">
@@ -10843,7 +10887,7 @@
         <v>354</v>
       </c>
       <c r="K61" s="15">
-        <f t="shared" ref="K61" si="11">I61</f>
+        <f>I61</f>
         <v>70211105</v>
       </c>
       <c r="L61" s="15" t="s">
@@ -10952,7 +10996,7 @@
         <v>364</v>
       </c>
       <c r="K63" s="15">
-        <f t="shared" ref="K63:K66" si="12">I63</f>
+        <f>I63</f>
         <v>70213008</v>
       </c>
       <c r="L63" s="15" t="s">
@@ -11007,7 +11051,7 @@
         <v>369</v>
       </c>
       <c r="K64" s="15">
-        <f t="shared" si="12"/>
+        <f>I64</f>
         <v>70211033</v>
       </c>
       <c r="L64" s="15" t="s">
@@ -11062,7 +11106,7 @@
         <v>374</v>
       </c>
       <c r="K65" s="15">
-        <f t="shared" si="12"/>
+        <f>I65</f>
         <v>70207015</v>
       </c>
       <c r="L65" s="15" t="s">
@@ -11117,7 +11161,7 @@
         <v>379</v>
       </c>
       <c r="K66" s="15">
-        <f t="shared" si="12"/>
+        <f>I66</f>
         <v>70212121</v>
       </c>
       <c r="L66" s="15" t="s">
@@ -11175,7 +11219,7 @@
         <v>70211110</v>
       </c>
       <c r="L67" s="14" t="s">
-        <v>211</v>
+        <v>73</v>
       </c>
       <c r="M67" s="14" t="b">
         <v>1</v>
@@ -11226,7 +11270,7 @@
         <v>386</v>
       </c>
       <c r="K68" s="15">
-        <f t="shared" ref="K68:K69" si="13">I68</f>
+        <f>I68</f>
         <v>70212073</v>
       </c>
       <c r="L68" s="15" t="s">
@@ -11281,7 +11325,7 @@
         <v>391</v>
       </c>
       <c r="K69" s="15">
-        <f t="shared" si="13"/>
+        <f>I69</f>
         <v>70211088</v>
       </c>
       <c r="L69" s="15" t="s">
@@ -11339,7 +11383,7 @@
         <v>70211242</v>
       </c>
       <c r="L70" s="15" t="s">
-        <v>211</v>
+        <v>80</v>
       </c>
       <c r="M70" s="15" t="b">
         <v>1</v>
@@ -11444,7 +11488,7 @@
         <v>405</v>
       </c>
       <c r="K72" s="15">
-        <f t="shared" ref="K72" si="14">I72</f>
+        <f>I72</f>
         <v>70214002</v>
       </c>
       <c r="L72" s="15" t="s">
@@ -11553,7 +11597,7 @@
         <v>411</v>
       </c>
       <c r="K74" s="15">
-        <f t="shared" ref="K74" si="15">I74</f>
+        <f>I74</f>
         <v>70222047</v>
       </c>
       <c r="L74" s="15" t="s">
@@ -11705,10 +11749,14 @@
       <c r="H77" s="14"/>
       <c r="I77" s="14"/>
       <c r="J77" s="14"/>
-      <c r="K77" s="15"/>
-      <c r="L77" s="15"/>
+      <c r="K77" s="24">
+        <v>70213038</v>
+      </c>
+      <c r="L77" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="M77" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N77" s="15"/>
       <c r="O77" s="16" t="s">
@@ -14385,7 +14433,7 @@
         <v>70211110</v>
       </c>
       <c r="L137" s="15" t="s">
-        <v>211</v>
+        <v>80</v>
       </c>
       <c r="M137" s="15" t="b">
         <v>1</v>
@@ -16123,7 +16171,7 @@
         <v>70211110</v>
       </c>
       <c r="L176" s="15" t="s">
-        <v>211</v>
+        <v>80</v>
       </c>
       <c r="M176" s="15" t="b">
         <v>1</v>

</xml_diff>